<commit_message>
Update data tables, scripts, and documentation
</commit_message>
<xml_diff>
--- a/data/trees/robustness_analyses.xlsx
+++ b/data/trees/robustness_analyses.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Eukaryotes_Asgard_TACK/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linweili/Important_files/课题进展/Asgard_Eukaryote_Data/data/trees/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6CB6B1F-A8F0-9B49-ADAF-FCC8E14B28CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19C4C65-FEE3-494E-BF8F-5EAD292AB805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="720" windowWidth="28040" windowHeight="17340" xr2:uid="{A8F32809-49F2-F649-AE47-172A25B57BE0}"/>
   </bookViews>
@@ -424,6 +424,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -449,12 +455,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -828,7 +828,7 @@
       <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="15" t="s">
         <v>39</v>
       </c>
     </row>
@@ -879,13 +879,13 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="17">
         <v>4740</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="17" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="5" t="s">
@@ -902,9 +902,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
       <c r="D6" s="8" t="s">
         <v>16</v>
       </c>
@@ -919,9 +919,9 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="5" t="s">
         <v>18</v>
       </c>
@@ -931,14 +931,14 @@
       <c r="F7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="25">
+      <c r="G7" s="16">
         <v>6.3600000000000001E-5</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="8" t="s">
         <v>20</v>
       </c>
@@ -953,9 +953,9 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
       <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
@@ -993,16 +993,16 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="17">
         <v>4740</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E11" s="10">
@@ -1016,10 +1016,10 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="11">
         <v>11443</v>
       </c>
@@ -1031,10 +1031,10 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
+      <c r="A13" s="21"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="10">
         <v>10636</v>
       </c>
@@ -1046,10 +1046,10 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="11">
         <v>12675</v>
       </c>
@@ -1061,10 +1061,10 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="10">
         <v>11350</v>
       </c>
@@ -1076,10 +1076,10 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="11">
         <v>11016</v>
       </c>
@@ -1091,10 +1091,10 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="10">
         <v>10894</v>
       </c>
@@ -1106,10 +1106,10 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
       <c r="E18" s="11">
         <v>10078</v>
       </c>
@@ -1121,10 +1121,10 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
       <c r="E19" s="10">
         <v>10096</v>
       </c>
@@ -1136,10 +1136,10 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
       <c r="E20" s="12">
         <v>10861</v>
       </c>

</xml_diff>